<commit_message>
Latest BOM comparision done.
BOM Abi final ni ha Client ki approvel abi ni ayi is lye.
</commit_message>
<xml_diff>
--- a/Deliverables/Bracelet(Main)/BOM/Bracelet_Main-PCB(Digikey).xlsx
+++ b/Deliverables/Bracelet(Main)/BOM/Bracelet_Main-PCB(Digikey).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Waqar\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Github\BrianPeri-SmartWatch\Deliverables\Bracelet(Main)\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB72D6C-E217-46B9-98FD-81ABEFC484BB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3EAF4F9-6D00-4AE0-8647-FF2CFE388350}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1810,6 +1810,15 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1817,6 +1826,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1824,21 +1839,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2145,25 +2145,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="115" t="s">
+      <c r="A1" s="110" t="s">
         <v>264</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="117"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="111"/>
+      <c r="J1" s="111"/>
+      <c r="K1" s="111"/>
+      <c r="L1" s="111"/>
+      <c r="M1" s="111"/>
+      <c r="N1" s="111"/>
+      <c r="O1" s="111"/>
+      <c r="P1" s="111"/>
+      <c r="Q1" s="112"/>
     </row>
     <row r="2" spans="1:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -2222,7 +2222,7 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="110" t="s">
+      <c r="B3" s="113" t="s">
         <v>247</v>
       </c>
       <c r="C3" s="44" t="s">
@@ -2276,7 +2276,7 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="111"/>
+      <c r="B4" s="114"/>
       <c r="C4" s="45" t="s">
         <v>8</v>
       </c>
@@ -2328,7 +2328,7 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="111"/>
+      <c r="B5" s="114"/>
       <c r="C5" s="45" t="s">
         <v>13</v>
       </c>
@@ -2380,7 +2380,7 @@
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="111"/>
+      <c r="B6" s="114"/>
       <c r="C6" s="46" t="s">
         <v>268</v>
       </c>
@@ -2432,7 +2432,7 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="111"/>
+      <c r="B7" s="114"/>
       <c r="C7" s="46" t="s">
         <v>269</v>
       </c>
@@ -2484,7 +2484,7 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="111"/>
+      <c r="B8" s="114"/>
       <c r="C8" s="45" t="s">
         <v>24</v>
       </c>
@@ -2536,7 +2536,7 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="111"/>
+      <c r="B9" s="114"/>
       <c r="C9" s="46" t="s">
         <v>270</v>
       </c>
@@ -2588,7 +2588,7 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="111"/>
+      <c r="B10" s="114"/>
       <c r="C10" s="46" t="s">
         <v>271</v>
       </c>
@@ -2640,7 +2640,7 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="111"/>
+      <c r="B11" s="114"/>
       <c r="C11" s="45" t="s">
         <v>34</v>
       </c>
@@ -2692,7 +2692,7 @@
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="112"/>
+      <c r="B12" s="115"/>
       <c r="C12" s="47" t="s">
         <v>38</v>
       </c>
@@ -2744,7 +2744,7 @@
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="118" t="s">
+      <c r="B13" s="116" t="s">
         <v>248</v>
       </c>
       <c r="C13" s="48" t="s">
@@ -2800,7 +2800,7 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="111"/>
+      <c r="B14" s="114"/>
       <c r="C14" s="45" t="s">
         <v>46</v>
       </c>
@@ -2854,7 +2854,7 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="119"/>
+      <c r="B15" s="117"/>
       <c r="C15" s="55" t="s">
         <v>275</v>
       </c>
@@ -2906,7 +2906,7 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="110" t="s">
+      <c r="B16" s="113" t="s">
         <v>249</v>
       </c>
       <c r="C16" s="60" t="s">
@@ -2962,7 +2962,7 @@
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="111"/>
+      <c r="B17" s="114"/>
       <c r="C17" s="49" t="s">
         <v>294</v>
       </c>
@@ -3016,7 +3016,7 @@
       <c r="A18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="111"/>
+      <c r="B18" s="114"/>
       <c r="C18" s="45" t="s">
         <v>69</v>
       </c>
@@ -3070,7 +3070,7 @@
       <c r="A19" s="1">
         <v>17</v>
       </c>
-      <c r="B19" s="112"/>
+      <c r="B19" s="115"/>
       <c r="C19" s="61" t="s">
         <v>276</v>
       </c>
@@ -3124,7 +3124,7 @@
       <c r="A20" s="1">
         <v>18</v>
       </c>
-      <c r="B20" s="118" t="s">
+      <c r="B20" s="116" t="s">
         <v>250</v>
       </c>
       <c r="C20" s="48" t="s">
@@ -3178,7 +3178,7 @@
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="119"/>
+      <c r="B21" s="117"/>
       <c r="C21" s="67" t="s">
         <v>87</v>
       </c>
@@ -3230,7 +3230,7 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="110" t="s">
+      <c r="B22" s="113" t="s">
         <v>251</v>
       </c>
       <c r="C22" s="69" t="s">
@@ -3284,7 +3284,7 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="111"/>
+      <c r="B23" s="114"/>
       <c r="C23" s="46" t="s">
         <v>281</v>
       </c>
@@ -3336,7 +3336,7 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="111"/>
+      <c r="B24" s="114"/>
       <c r="C24" s="46" t="s">
         <v>280</v>
       </c>
@@ -3388,7 +3388,7 @@
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="111"/>
+      <c r="B25" s="114"/>
       <c r="C25" s="46" t="s">
         <v>282</v>
       </c>
@@ -3440,7 +3440,7 @@
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="111"/>
+      <c r="B26" s="114"/>
       <c r="C26" s="46" t="s">
         <v>283</v>
       </c>
@@ -3492,7 +3492,7 @@
       <c r="A27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" s="111"/>
+      <c r="B27" s="114"/>
       <c r="C27" s="45" t="s">
         <v>107</v>
       </c>
@@ -3544,7 +3544,7 @@
       <c r="A28" s="1">
         <v>26</v>
       </c>
-      <c r="B28" s="111"/>
+      <c r="B28" s="114"/>
       <c r="C28" s="46" t="s">
         <v>284</v>
       </c>
@@ -3596,7 +3596,7 @@
       <c r="A29" s="1">
         <v>27</v>
       </c>
-      <c r="B29" s="111"/>
+      <c r="B29" s="114"/>
       <c r="C29" s="46" t="s">
         <v>285</v>
       </c>
@@ -3648,7 +3648,7 @@
       <c r="A30" s="1">
         <v>28</v>
       </c>
-      <c r="B30" s="111"/>
+      <c r="B30" s="114"/>
       <c r="C30" s="46" t="s">
         <v>286</v>
       </c>
@@ -3700,7 +3700,7 @@
       <c r="A31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" s="111"/>
+      <c r="B31" s="114"/>
       <c r="C31" s="45" t="s">
         <v>120</v>
       </c>
@@ -3752,7 +3752,7 @@
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" s="111"/>
+      <c r="B32" s="114"/>
       <c r="C32" s="46" t="s">
         <v>287</v>
       </c>
@@ -3804,7 +3804,7 @@
       <c r="A33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" s="111"/>
+      <c r="B33" s="114"/>
       <c r="C33" s="45" t="s">
         <v>126</v>
       </c>
@@ -3856,7 +3856,7 @@
       <c r="A34" s="1">
         <v>32</v>
       </c>
-      <c r="B34" s="112"/>
+      <c r="B34" s="115"/>
       <c r="C34" s="61" t="s">
         <v>288</v>
       </c>
@@ -4018,7 +4018,7 @@
       <c r="A37" s="1">
         <v>35</v>
       </c>
-      <c r="B37" s="110" t="s">
+      <c r="B37" s="113" t="s">
         <v>254</v>
       </c>
       <c r="C37" s="60" t="s">
@@ -4074,7 +4074,7 @@
       <c r="A38" s="1">
         <v>36</v>
       </c>
-      <c r="B38" s="111"/>
+      <c r="B38" s="114"/>
       <c r="C38" s="45" t="s">
         <v>295</v>
       </c>
@@ -4126,7 +4126,7 @@
       <c r="A39" s="1">
         <v>37</v>
       </c>
-      <c r="B39" s="111"/>
+      <c r="B39" s="114"/>
       <c r="C39" s="45" t="s">
         <v>146</v>
       </c>
@@ -4180,7 +4180,7 @@
       <c r="A40" s="1">
         <v>38</v>
       </c>
-      <c r="B40" s="111"/>
+      <c r="B40" s="114"/>
       <c r="C40" s="45" t="s">
         <v>150</v>
       </c>
@@ -4234,7 +4234,7 @@
       <c r="A41" s="1">
         <v>39</v>
       </c>
-      <c r="B41" s="111"/>
+      <c r="B41" s="114"/>
       <c r="C41" s="45" t="s">
         <v>154</v>
       </c>
@@ -4288,7 +4288,7 @@
       <c r="A42" s="1">
         <v>40</v>
       </c>
-      <c r="B42" s="111"/>
+      <c r="B42" s="114"/>
       <c r="C42" s="45" t="s">
         <v>297</v>
       </c>
@@ -4342,7 +4342,7 @@
       <c r="A43" s="1">
         <v>41</v>
       </c>
-      <c r="B43" s="111"/>
+      <c r="B43" s="114"/>
       <c r="C43" s="45" t="s">
         <v>161</v>
       </c>
@@ -4396,7 +4396,7 @@
       <c r="A44" s="1">
         <v>42</v>
       </c>
-      <c r="B44" s="111"/>
+      <c r="B44" s="114"/>
       <c r="C44" s="45" t="s">
         <v>165</v>
       </c>
@@ -4450,7 +4450,7 @@
       <c r="A45" s="1">
         <v>43</v>
       </c>
-      <c r="B45" s="112"/>
+      <c r="B45" s="115"/>
       <c r="C45" s="70" t="s">
         <v>169</v>
       </c>
@@ -4502,7 +4502,7 @@
       <c r="A46" s="1">
         <v>44</v>
       </c>
-      <c r="B46" s="110" t="s">
+      <c r="B46" s="113" t="s">
         <v>255</v>
       </c>
       <c r="C46" s="60" t="s">
@@ -4558,7 +4558,7 @@
       <c r="A47" s="1">
         <v>45</v>
       </c>
-      <c r="B47" s="111"/>
+      <c r="B47" s="114"/>
       <c r="C47" s="45" t="s">
         <v>296</v>
       </c>
@@ -4612,7 +4612,7 @@
       <c r="A48" s="1">
         <v>46</v>
       </c>
-      <c r="B48" s="111"/>
+      <c r="B48" s="114"/>
       <c r="C48" s="45" t="s">
         <v>58</v>
       </c>
@@ -4664,7 +4664,7 @@
       <c r="A49" s="1">
         <v>47</v>
       </c>
-      <c r="B49" s="111"/>
+      <c r="B49" s="114"/>
       <c r="C49" s="45" t="s">
         <v>52</v>
       </c>
@@ -4716,7 +4716,7 @@
       <c r="A50" s="1">
         <v>48</v>
       </c>
-      <c r="B50" s="111"/>
+      <c r="B50" s="114"/>
       <c r="C50" s="45" t="s">
         <v>55</v>
       </c>
@@ -4768,7 +4768,7 @@
       <c r="A51" s="1">
         <v>49</v>
       </c>
-      <c r="B51" s="111"/>
+      <c r="B51" s="114"/>
       <c r="C51" s="45" t="s">
         <v>79</v>
       </c>
@@ -4820,7 +4820,7 @@
       <c r="A52" s="1">
         <v>50</v>
       </c>
-      <c r="B52" s="112"/>
+      <c r="B52" s="115"/>
       <c r="C52" s="89" t="s">
         <v>133</v>
       </c>
@@ -4943,24 +4943,24 @@
       </c>
     </row>
     <row r="55" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J55" s="113" t="s">
+      <c r="J55" s="118" t="s">
         <v>262</v>
       </c>
-      <c r="K55" s="113"/>
-      <c r="L55" s="113"/>
-      <c r="M55" s="113"/>
+      <c r="K55" s="118"/>
+      <c r="L55" s="118"/>
+      <c r="M55" s="118"/>
       <c r="P55" s="19">
         <f>SUM(P3:P47)</f>
         <v>247.77164999999997</v>
       </c>
     </row>
     <row r="56" spans="1:17" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="J56" s="114" t="s">
+      <c r="J56" s="119" t="s">
         <v>263</v>
       </c>
-      <c r="K56" s="114"/>
-      <c r="L56" s="114"/>
-      <c r="M56" s="114"/>
+      <c r="K56" s="119"/>
+      <c r="L56" s="119"/>
+      <c r="M56" s="119"/>
       <c r="N56" s="18">
         <f>SUM(N3:N47)</f>
         <v>53.327129999999997</v>
@@ -4972,16 +4972,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B22:B34"/>
+    <mergeCell ref="B37:B45"/>
+    <mergeCell ref="B46:B52"/>
+    <mergeCell ref="J55:M55"/>
+    <mergeCell ref="J56:M56"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="B3:B12"/>
     <mergeCell ref="B13:B15"/>
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B22:B34"/>
-    <mergeCell ref="B37:B45"/>
-    <mergeCell ref="B46:B52"/>
-    <mergeCell ref="J55:M55"/>
-    <mergeCell ref="J56:M56"/>
   </mergeCells>
   <conditionalFormatting sqref="N56:P56">
     <cfRule type="dataBar" priority="5">

</xml_diff>